<commit_message>
feat(quan-ly): cập nhật file Excel có biểu đồ và công thức mới
</commit_message>
<xml_diff>
--- a/quan-ly-du-an/phan-tich-bai-bao.xlsx
+++ b/quan-ly-du-an/phan-tich-bai-bao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Esclipe_Web\Quan ly du an HTTT\quan-ly-du-an\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC753A5F-E294-4479-B187-C312CC1EC8C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580DC734-C9F1-44FC-A08A-B99672C6B73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1848" yWindow="1848" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -920,7 +920,7 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="1"/>
+      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1028,7 +1028,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F044-42C7-BA77-2BE68DD3C94C}"/>
+              <c16:uniqueId val="{00000000-D452-46D1-BF3D-81C9AB73AA34}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1131,7 +1131,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-F044-42C7-BA77-2BE68DD3C94C}"/>
+              <c16:uniqueId val="{00000001-D452-46D1-BF3D-81C9AB73AA34}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1152,7 +1152,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1172,26 +1172,9 @@
           <c:max val="1"/>
           <c:min val="0"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:majorGridlines/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>RII</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="1"/>
-        </c:title>
         <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1202,8 +1185,8 @@
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="1"/>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
@@ -1239,7 +1222,7 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="1"/>
+      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1371,7 +1354,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1726-4066-84CE-E1B6A2C58305}"/>
+              <c16:uniqueId val="{00000000-5734-423D-857B-709CF20B09FA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1498,7 +1481,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1726-4066-84CE-E1B6A2C58305}"/>
+              <c16:uniqueId val="{00000001-5734-423D-857B-709CF20B09FA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1519,7 +1502,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1539,26 +1522,9 @@
           <c:max val="0.9"/>
           <c:min val="0.4"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>AVE</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="1"/>
-        </c:title>
         <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1569,8 +1535,8 @@
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="1"/>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
@@ -1606,7 +1572,7 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="1"/>
+      <c:overlay val="0"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1732,7 +1698,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A5C4-43B1-A5BE-36E2F67D9E98}"/>
+              <c16:uniqueId val="{00000000-6524-4F3A-8354-A2DF737ECD18}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1853,7 +1819,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A5C4-43B1-A5BE-36E2F67D9E98}"/>
+              <c16:uniqueId val="{00000001-6524-4F3A-8354-A2DF737ECD18}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1874,7 +1840,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1892,26 +1858,9 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Hệ số</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="1"/>
-        </c:title>
         <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1922,8 +1871,8 @@
       </c:valAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="1"/>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>

</xml_diff>